<commit_message>
feat: add instagram logos (round static and animated pointer)
</commit_message>
<xml_diff>
--- a/telegram_brand_emojis_registry.xlsx
+++ b/telegram_brand_emojis_registry.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -874,6 +874,86 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>لوگو اینستاگرام گرد</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>شبکه‌های اجتماعی / لینک‌ها</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>LogoandDesign</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>🟣</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>5375401795738682827</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>&lt;tg-emoji emoji-id="5375401795738682827"&gt;🟣&lt;/tg-emoji&gt;</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>icon_custom_emoji_id="5375401795738682827"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>آیکون اینستاگرام با اشاره‌گر به راست (متحرک)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>شبکه‌های اجتماعی / دکمه لینک</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Mega_Logo</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>🌐</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>5384234065270433395</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>&lt;tg-emoji emoji-id="5384234065270433395"&gt;🌐&lt;/tg-emoji&gt;</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>icon_custom_emoji_id="5384234065270433395"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add animated trash bin custom emoji
</commit_message>
<xml_diff>
--- a/telegram_brand_emojis_registry.xlsx
+++ b/telegram_brand_emojis_registry.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -954,6 +954,46 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>سطل آشغال (حذف / پاک کردن - متحرک)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>عملیات / سبد خرید و مدیریت</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>NewsEmoji</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>🗑</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>5445267414562389170</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>&lt;tg-emoji emoji-id="5445267414562389170"&gt;🗑&lt;/tg-emoji&gt;</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>icon_custom_emoji_id="5445267414562389170"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add animated search icon
</commit_message>
<xml_diff>
--- a/telegram_brand_emojis_registry.xlsx
+++ b/telegram_brand_emojis_registry.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -994,6 +994,46 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>جستجو / سرچ کاتالوگ (متحرک)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>ناوبری / جستجو و فیلتر</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>KorysnostiDevicesIcons</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>📄</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>5431420628978641216</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>&lt;tg-emoji emoji-id="5431420628978641216"&gt;📄&lt;/tg-emoji&gt;</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>icon_custom_emoji_id="5431420628978641216"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add animated persian support icon
</commit_message>
<xml_diff>
--- a/telegram_brand_emojis_registry.xlsx
+++ b/telegram_brand_emojis_registry.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1034,6 +1034,46 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>استیکر متحرک پشتیبانی با متن فارسی</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>پشتیبانی / ارتباط با ادمین</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>propiycom</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>💵</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>5958416857114350105</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>&lt;tg-emoji emoji-id="5958416857114350105"&gt;💵&lt;/tg-emoji&gt;</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>icon_custom_emoji_id="5958416857114350105"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>